<commit_message>
chore: sync SALEC audit hardening and dev setup to NEW_PRO baseline
Includes security/infra refactors, docs, CI workflows, and local Docker env wiring without committing secrets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/audit-output/expeditor-smoke/ex-2.0.xlsx
+++ b/backend/scripts/audit-output/expeditor-smoke/ex-2.0.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="110">
-  <si>
-    <t>Загрузочный лист 2.0 (Время печати: 27.05.2026 19:51:40)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+  <si>
+    <t>Загрузочный лист 2.0 (Время печати: 28.05.2026 17:37:19)</t>
   </si>
   <si>
     <t>LIPUCHKA</t>
@@ -779,15 +779,15 @@
     <pageSetUpPr fitToPage="1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AD44"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <dimension ref="A1:AN44"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -829,7 +829,7 @@
       </c>
       <c r="X1" s="5"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
@@ -895,7 +895,7 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
@@ -925,7 +925,7 @@
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>30</v>
       </c>
@@ -955,7 +955,7 @@
       <c r="W4" s="5"/>
       <c r="X4" s="5"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>32</v>
       </c>
@@ -985,7 +985,7 @@
       <c r="W5" s="5"/>
       <c r="X5" s="5"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>34</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>37</v>
       </c>
@@ -2320,6 +2320,6 @@
     <mergeCell ref="A44:C44"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>